<commit_message>
fix: Self Assessment file corrected
</commit_message>
<xml_diff>
--- a/scrum/TeamSelfAssessment/sprint3/SEM3-PI2526-SA-G052-Sprint3.xlsx
+++ b/scrum/TeamSelfAssessment/sprint3/SEM3-PI2526-SA-G052-Sprint3.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gonca\IdeaProjects\sem3-pi-25-26-g052-repo\scrum\TeamSelfAssessment\sprint3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85E312C2-0C8B-4CDC-99CD-8F41F7644723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{307BE121-E816-41F5-985D-6C64C48ACEA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Team and Self Assessment" sheetId="2" r:id="rId1"/>
-    <sheet name="User Stories-not-mandatory" sheetId="5" r:id="rId2"/>
+    <sheet name="User Stories-Mandatory" sheetId="5" r:id="rId2"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId3"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="75">
   <si>
     <t>TeamID #</t>
   </si>
@@ -156,15 +156,9 @@
     <t>Assessment weight:</t>
   </si>
   <si>
-    <t>User Manual (LAPR2)</t>
-  </si>
-  <si>
     <t>Write the student name and number in Column C (team members).</t>
   </si>
   <si>
-    <t>Student Name &amp; Number 6</t>
-  </si>
-  <si>
     <t>Student Name &amp; Number 7</t>
   </si>
   <si>
@@ -196,6 +190,96 @@
   </si>
   <si>
     <t>LAPR3 Project: Team and Self-assessment    SPRINT 2</t>
+  </si>
+  <si>
+    <t>ALL</t>
+  </si>
+  <si>
+    <t>USEI11</t>
+  </si>
+  <si>
+    <t>The US was implemented as asked, meeting all the requirements</t>
+  </si>
+  <si>
+    <t>UESEI12</t>
+  </si>
+  <si>
+    <t>USEI13</t>
+  </si>
+  <si>
+    <t>USEI14</t>
+  </si>
+  <si>
+    <t>USEI15</t>
+  </si>
+  <si>
+    <t>USAC10</t>
+  </si>
+  <si>
+    <t>USAC11</t>
+  </si>
+  <si>
+    <t>USAC12</t>
+  </si>
+  <si>
+    <t>USAC13</t>
+  </si>
+  <si>
+    <t>USAC14</t>
+  </si>
+  <si>
+    <t>USAC15</t>
+  </si>
+  <si>
+    <t>USAC16</t>
+  </si>
+  <si>
+    <t>USLP8</t>
+  </si>
+  <si>
+    <t>USLP9</t>
+  </si>
+  <si>
+    <t>USLP10</t>
+  </si>
+  <si>
+    <t>USBD31</t>
+  </si>
+  <si>
+    <t>USBD32</t>
+  </si>
+  <si>
+    <t>USBD33</t>
+  </si>
+  <si>
+    <t>USBD34</t>
+  </si>
+  <si>
+    <t>USBD35</t>
+  </si>
+  <si>
+    <t>USBD36</t>
+  </si>
+  <si>
+    <t>USBD37</t>
+  </si>
+  <si>
+    <t>USBD39</t>
+  </si>
+  <si>
+    <t>USBD41</t>
+  </si>
+  <si>
+    <t>USBD42</t>
+  </si>
+  <si>
+    <t>USBD43</t>
+  </si>
+  <si>
+    <t>USBD44</t>
+  </si>
+  <si>
+    <t>USBD45</t>
   </si>
 </sst>
 </file>
@@ -250,7 +334,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -281,8 +365,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="35">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -443,19 +533,6 @@
         <color indexed="64"/>
       </top>
       <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -742,7 +819,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -781,13 +858,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -797,83 +874,77 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="65" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="65" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="65" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="65" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="24" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="34" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
@@ -885,32 +956,45 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1449,14 +1533,14 @@
   <sheetData>
     <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="17" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.5">
-      <c r="A2" s="23" t="s">
-        <v>38</v>
+      <c r="A2" s="22" t="s">
+        <v>36</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1485,99 +1569,99 @@
     <row r="8" spans="1:13" ht="15.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
-      <c r="E8" s="60" t="s">
+      <c r="E8" s="58" t="s">
         <v>3</v>
       </c>
-      <c r="F8" s="61"/>
-      <c r="G8" s="61"/>
-      <c r="H8" s="61"/>
-      <c r="I8" s="61"/>
-      <c r="J8" s="61"/>
-      <c r="K8" s="61"/>
-      <c r="L8" s="61"/>
-      <c r="M8" s="62"/>
+      <c r="F8" s="59"/>
+      <c r="G8" s="59"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="59"/>
+      <c r="J8" s="59"/>
+      <c r="K8" s="59"/>
+      <c r="L8" s="59"/>
+      <c r="M8" s="60"/>
     </row>
     <row r="9" spans="1:13" ht="105.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
-      <c r="D9" s="29" t="str">
+      <c r="D9" s="28" t="str">
         <f>C10</f>
         <v>Francisco Vasconcelos 1240934</v>
       </c>
-      <c r="E9" s="30" t="str">
+      <c r="E9" s="29" t="str">
         <f>C11</f>
         <v>Gabriel Inácio 1240935</v>
       </c>
-      <c r="F9" s="30" t="str">
+      <c r="F9" s="29" t="str">
         <f>C12</f>
         <v>Gonçalo Azevedo 1240936</v>
       </c>
-      <c r="G9" s="30" t="str">
+      <c r="G9" s="29" t="str">
         <f>C13</f>
         <v>Maria Pinto 1240892</v>
       </c>
-      <c r="H9" s="30" t="str">
+      <c r="H9" s="29" t="str">
         <f>C14</f>
         <v>Paulo Ferreira 1240941</v>
       </c>
-      <c r="I9" s="30" t="str">
+      <c r="I9" s="29" t="str">
         <f>C15</f>
-        <v>Student Name &amp; Number 6</v>
-      </c>
-      <c r="J9" s="30" t="str">
+        <v>ALL</v>
+      </c>
+      <c r="J9" s="29" t="str">
         <f>C16</f>
         <v>Student Name &amp; Number 7</v>
       </c>
-      <c r="K9" s="30" t="str">
+      <c r="K9" s="29" t="str">
         <f>C17</f>
         <v>Student Name &amp; Number 8</v>
       </c>
-      <c r="L9" s="31" t="s">
+      <c r="L9" s="30" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B10" s="57" t="s">
+      <c r="B10" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="25" t="s">
-        <v>41</v>
-      </c>
-      <c r="D10" s="53">
+      <c r="C10" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="51">
         <v>5</v>
       </c>
-      <c r="E10" s="26">
-        <v>4</v>
-      </c>
-      <c r="F10" s="27">
+      <c r="E10" s="25">
+        <v>4</v>
+      </c>
+      <c r="F10" s="26">
         <v>5</v>
       </c>
-      <c r="G10" s="27">
+      <c r="G10" s="26">
         <v>5</v>
       </c>
-      <c r="H10" s="27">
+      <c r="H10" s="26">
         <v>5</v>
       </c>
-      <c r="I10" s="27"/>
-      <c r="J10" s="27"/>
-      <c r="K10" s="25"/>
-      <c r="L10" s="35">
+      <c r="I10" s="26"/>
+      <c r="J10" s="26"/>
+      <c r="K10" s="24"/>
+      <c r="L10" s="34">
         <f t="shared" ref="L10:L17" si="0">AVERAGE(D10:K10)</f>
         <v>4.8</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="31.9" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B11" s="58"/>
+      <c r="B11" s="56"/>
       <c r="C11" s="6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D11" s="7">
         <v>4</v>
       </c>
-      <c r="E11" s="53">
-        <v>4</v>
-      </c>
-      <c r="F11" s="24">
+      <c r="E11" s="51">
+        <v>4</v>
+      </c>
+      <c r="F11" s="23">
         <v>4</v>
       </c>
       <c r="G11" s="6">
@@ -1589,15 +1673,15 @@
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
       <c r="K11" s="8"/>
-      <c r="L11" s="36">
+      <c r="L11" s="35">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B12" s="58"/>
+      <c r="B12" s="56"/>
       <c r="C12" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D12" s="6">
         <v>5</v>
@@ -1605,10 +1689,10 @@
       <c r="E12" s="7">
         <v>4</v>
       </c>
-      <c r="F12" s="53">
+      <c r="F12" s="51">
         <v>5</v>
       </c>
-      <c r="G12" s="24">
+      <c r="G12" s="23">
         <v>5</v>
       </c>
       <c r="H12" s="6">
@@ -1617,15 +1701,15 @@
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
       <c r="K12" s="8"/>
-      <c r="L12" s="36">
+      <c r="L12" s="35">
         <f t="shared" si="0"/>
         <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="31.9" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B13" s="58"/>
+      <c r="B13" s="56"/>
       <c r="C13" s="6" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D13" s="6">
         <v>5</v>
@@ -1636,24 +1720,24 @@
       <c r="F13" s="7">
         <v>5</v>
       </c>
-      <c r="G13" s="53">
+      <c r="G13" s="51">
         <v>5</v>
       </c>
-      <c r="H13" s="56">
+      <c r="H13" s="54">
         <v>5</v>
       </c>
       <c r="I13" s="6"/>
       <c r="J13" s="6"/>
       <c r="K13" s="8"/>
-      <c r="L13" s="36">
+      <c r="L13" s="35">
         <f t="shared" si="0"/>
         <v>4.8</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="31.9" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B14" s="58"/>
+      <c r="B14" s="56"/>
       <c r="C14" s="6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D14" s="6">
         <v>5</v>
@@ -1667,39 +1751,39 @@
       <c r="G14" s="7">
         <v>5</v>
       </c>
-      <c r="H14" s="53">
+      <c r="H14" s="51">
         <v>5</v>
       </c>
-      <c r="I14" s="24"/>
+      <c r="I14" s="23"/>
       <c r="J14" s="6"/>
       <c r="K14" s="8"/>
-      <c r="L14" s="36">
+      <c r="L14" s="35">
         <f t="shared" si="0"/>
         <v>4.8</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="31.9" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B15" s="58"/>
+    <row r="15" spans="1:13" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B15" s="56"/>
       <c r="C15" s="6" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
       <c r="G15" s="6"/>
       <c r="H15" s="7"/>
-      <c r="I15" s="53"/>
-      <c r="J15" s="24"/>
+      <c r="I15" s="51"/>
+      <c r="J15" s="23"/>
       <c r="K15" s="8"/>
-      <c r="L15" s="36" t="e">
+      <c r="L15" s="35" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="31.9" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B16" s="58"/>
+      <c r="B16" s="56"/>
       <c r="C16" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
@@ -1707,285 +1791,285 @@
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
       <c r="I16" s="7"/>
-      <c r="J16" s="53"/>
+      <c r="J16" s="51"/>
       <c r="K16" s="8"/>
-      <c r="L16" s="36" t="e">
+      <c r="L16" s="35" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="31.9" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B17" s="59"/>
+      <c r="B17" s="57"/>
       <c r="C17" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28"/>
-      <c r="F17" s="28"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="28"/>
-      <c r="I17" s="28"/>
-      <c r="J17" s="28"/>
-      <c r="K17" s="54"/>
-      <c r="L17" s="37" t="e">
+        <v>35</v>
+      </c>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="27"/>
+      <c r="J17" s="27"/>
+      <c r="K17" s="52"/>
+      <c r="L17" s="36" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="18" spans="1:12" ht="31.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" s="1"/>
-      <c r="C18" s="32" t="s">
-        <v>39</v>
-      </c>
-      <c r="D18" s="33">
+      <c r="C18" s="31" t="s">
+        <v>37</v>
+      </c>
+      <c r="D18" s="32">
         <f t="shared" ref="D18:K18" si="1">AVERAGE(D10:D17)</f>
         <v>4.8</v>
       </c>
-      <c r="E18" s="33">
+      <c r="E18" s="32">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="F18" s="33">
+      <c r="F18" s="32">
         <f t="shared" si="1"/>
         <v>4.8</v>
       </c>
-      <c r="G18" s="33">
+      <c r="G18" s="32">
         <f t="shared" si="1"/>
         <v>4.8</v>
       </c>
-      <c r="H18" s="33">
+      <c r="H18" s="32">
         <f t="shared" si="1"/>
         <v>4.5999999999999996</v>
       </c>
-      <c r="I18" s="33" t="e">
+      <c r="I18" s="32" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="J18" s="33" t="e">
+      <c r="J18" s="32" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="K18" s="34" t="e">
+      <c r="K18" s="33" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="L18" s="38"/>
+      <c r="L18" s="37"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A20" s="42" t="s">
+      <c r="A20" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="43"/>
-      <c r="C20" s="43"/>
-      <c r="D20" s="43"/>
-      <c r="E20" s="43"/>
-      <c r="F20" s="43"/>
-      <c r="G20" s="43"/>
-      <c r="H20" s="43"/>
-      <c r="I20" s="43"/>
-      <c r="J20" s="43"/>
-      <c r="K20" s="43"/>
-      <c r="L20" s="44"/>
+      <c r="B20" s="41"/>
+      <c r="C20" s="41"/>
+      <c r="D20" s="41"/>
+      <c r="E20" s="41"/>
+      <c r="F20" s="41"/>
+      <c r="G20" s="41"/>
+      <c r="H20" s="41"/>
+      <c r="I20" s="41"/>
+      <c r="J20" s="41"/>
+      <c r="K20" s="41"/>
+      <c r="L20" s="42"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A21" s="45" t="s">
-        <v>34</v>
-      </c>
-      <c r="B21" s="46"/>
-      <c r="C21" s="46"/>
-      <c r="D21" s="46"/>
-      <c r="E21" s="46"/>
-      <c r="F21" s="46"/>
-      <c r="G21" s="46"/>
-      <c r="H21" s="46"/>
-      <c r="I21" s="46"/>
-      <c r="J21" s="46"/>
-      <c r="K21" s="46"/>
-      <c r="L21" s="47"/>
+      <c r="A21" s="43" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" s="44"/>
+      <c r="C21" s="44"/>
+      <c r="D21" s="44"/>
+      <c r="E21" s="44"/>
+      <c r="F21" s="44"/>
+      <c r="G21" s="44"/>
+      <c r="H21" s="44"/>
+      <c r="I21" s="44"/>
+      <c r="J21" s="44"/>
+      <c r="K21" s="44"/>
+      <c r="L21" s="45"/>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A22" s="48" t="s">
+      <c r="A22" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="B22" s="46"/>
-      <c r="C22" s="46"/>
-      <c r="D22" s="46"/>
-      <c r="E22" s="46"/>
-      <c r="F22" s="46"/>
-      <c r="G22" s="46"/>
-      <c r="H22" s="46"/>
-      <c r="I22" s="46"/>
-      <c r="J22" s="46"/>
-      <c r="K22" s="46"/>
-      <c r="L22" s="47"/>
+      <c r="B22" s="44"/>
+      <c r="C22" s="44"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="44"/>
+      <c r="F22" s="44"/>
+      <c r="G22" s="44"/>
+      <c r="H22" s="44"/>
+      <c r="I22" s="44"/>
+      <c r="J22" s="44"/>
+      <c r="K22" s="44"/>
+      <c r="L22" s="45"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A23" s="55" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23" s="46"/>
-      <c r="C23" s="46"/>
-      <c r="D23" s="46"/>
-      <c r="E23" s="46"/>
-      <c r="F23" s="46"/>
-      <c r="G23" s="46"/>
-      <c r="H23" s="46"/>
-      <c r="I23" s="46"/>
-      <c r="J23" s="46"/>
-      <c r="K23" s="46"/>
-      <c r="L23" s="47"/>
+      <c r="A23" s="53" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" s="44"/>
+      <c r="C23" s="44"/>
+      <c r="D23" s="44"/>
+      <c r="E23" s="44"/>
+      <c r="F23" s="44"/>
+      <c r="G23" s="44"/>
+      <c r="H23" s="44"/>
+      <c r="I23" s="44"/>
+      <c r="J23" s="44"/>
+      <c r="K23" s="44"/>
+      <c r="L23" s="45"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A24" s="45"/>
-      <c r="B24" s="46"/>
-      <c r="C24" s="46"/>
-      <c r="D24" s="46"/>
-      <c r="E24" s="46"/>
-      <c r="F24" s="46"/>
-      <c r="G24" s="46"/>
-      <c r="H24" s="46"/>
-      <c r="I24" s="46"/>
-      <c r="J24" s="46"/>
-      <c r="K24" s="46"/>
-      <c r="L24" s="47"/>
+      <c r="A24" s="43"/>
+      <c r="B24" s="44"/>
+      <c r="C24" s="44"/>
+      <c r="D24" s="44"/>
+      <c r="E24" s="44"/>
+      <c r="F24" s="44"/>
+      <c r="G24" s="44"/>
+      <c r="H24" s="44"/>
+      <c r="I24" s="44"/>
+      <c r="J24" s="44"/>
+      <c r="K24" s="44"/>
+      <c r="L24" s="45"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A25" s="49" t="s">
+      <c r="A25" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="B25" s="46"/>
-      <c r="C25" s="46"/>
-      <c r="D25" s="46"/>
-      <c r="E25" s="46"/>
-      <c r="F25" s="46"/>
-      <c r="G25" s="46"/>
-      <c r="H25" s="46"/>
-      <c r="I25" s="46"/>
-      <c r="J25" s="46"/>
-      <c r="K25" s="46"/>
-      <c r="L25" s="47"/>
+      <c r="B25" s="44"/>
+      <c r="C25" s="44"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="44"/>
+      <c r="F25" s="44"/>
+      <c r="G25" s="44"/>
+      <c r="H25" s="44"/>
+      <c r="I25" s="44"/>
+      <c r="J25" s="44"/>
+      <c r="K25" s="44"/>
+      <c r="L25" s="45"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A26" s="45">
+      <c r="A26" s="43">
         <v>0</v>
       </c>
-      <c r="B26" s="46" t="s">
+      <c r="B26" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="C26" s="46"/>
-      <c r="D26" s="46"/>
-      <c r="E26" s="46"/>
-      <c r="F26" s="46"/>
-      <c r="G26" s="46"/>
-      <c r="H26" s="46"/>
-      <c r="I26" s="46"/>
-      <c r="J26" s="46"/>
-      <c r="K26" s="46"/>
-      <c r="L26" s="47"/>
+      <c r="C26" s="44"/>
+      <c r="D26" s="44"/>
+      <c r="E26" s="44"/>
+      <c r="F26" s="44"/>
+      <c r="G26" s="44"/>
+      <c r="H26" s="44"/>
+      <c r="I26" s="44"/>
+      <c r="J26" s="44"/>
+      <c r="K26" s="44"/>
+      <c r="L26" s="45"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A27" s="45">
+      <c r="A27" s="43">
         <v>1</v>
       </c>
-      <c r="B27" s="46" t="s">
+      <c r="B27" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="C27" s="46"/>
-      <c r="D27" s="46"/>
-      <c r="E27" s="46"/>
-      <c r="F27" s="46"/>
-      <c r="G27" s="46"/>
-      <c r="H27" s="46"/>
-      <c r="I27" s="46"/>
-      <c r="J27" s="46"/>
-      <c r="K27" s="46"/>
-      <c r="L27" s="47"/>
+      <c r="C27" s="44"/>
+      <c r="D27" s="44"/>
+      <c r="E27" s="44"/>
+      <c r="F27" s="44"/>
+      <c r="G27" s="44"/>
+      <c r="H27" s="44"/>
+      <c r="I27" s="44"/>
+      <c r="J27" s="44"/>
+      <c r="K27" s="44"/>
+      <c r="L27" s="45"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A28" s="45">
+      <c r="A28" s="43">
         <v>2</v>
       </c>
-      <c r="B28" s="46" t="s">
+      <c r="B28" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="C28" s="46"/>
-      <c r="D28" s="46"/>
-      <c r="E28" s="46"/>
-      <c r="F28" s="46"/>
-      <c r="G28" s="46"/>
-      <c r="H28" s="46"/>
-      <c r="I28" s="46"/>
-      <c r="J28" s="46"/>
-      <c r="K28" s="46"/>
-      <c r="L28" s="47"/>
+      <c r="C28" s="44"/>
+      <c r="D28" s="44"/>
+      <c r="E28" s="44"/>
+      <c r="F28" s="44"/>
+      <c r="G28" s="44"/>
+      <c r="H28" s="44"/>
+      <c r="I28" s="44"/>
+      <c r="J28" s="44"/>
+      <c r="K28" s="44"/>
+      <c r="L28" s="45"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A29" s="45">
+      <c r="A29" s="43">
         <v>3</v>
       </c>
-      <c r="B29" s="46" t="s">
+      <c r="B29" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="C29" s="46"/>
-      <c r="D29" s="46"/>
-      <c r="E29" s="46"/>
-      <c r="F29" s="46"/>
-      <c r="G29" s="46"/>
-      <c r="H29" s="46"/>
-      <c r="I29" s="46"/>
-      <c r="J29" s="46"/>
-      <c r="K29" s="46"/>
-      <c r="L29" s="47"/>
+      <c r="C29" s="44"/>
+      <c r="D29" s="44"/>
+      <c r="E29" s="44"/>
+      <c r="F29" s="44"/>
+      <c r="G29" s="44"/>
+      <c r="H29" s="44"/>
+      <c r="I29" s="44"/>
+      <c r="J29" s="44"/>
+      <c r="K29" s="44"/>
+      <c r="L29" s="45"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A30" s="45">
-        <v>4</v>
-      </c>
-      <c r="B30" s="46" t="s">
+      <c r="A30" s="43">
+        <v>4</v>
+      </c>
+      <c r="B30" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="C30" s="46"/>
-      <c r="D30" s="46"/>
-      <c r="E30" s="46"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="46"/>
-      <c r="H30" s="46"/>
-      <c r="I30" s="46"/>
-      <c r="J30" s="46"/>
-      <c r="K30" s="46"/>
-      <c r="L30" s="47"/>
+      <c r="C30" s="44"/>
+      <c r="D30" s="44"/>
+      <c r="E30" s="44"/>
+      <c r="F30" s="44"/>
+      <c r="G30" s="44"/>
+      <c r="H30" s="44"/>
+      <c r="I30" s="44"/>
+      <c r="J30" s="44"/>
+      <c r="K30" s="44"/>
+      <c r="L30" s="45"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A31" s="45">
+      <c r="A31" s="43">
         <v>5</v>
       </c>
-      <c r="B31" s="46" t="s">
+      <c r="B31" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="C31" s="46"/>
-      <c r="D31" s="46"/>
-      <c r="E31" s="46"/>
-      <c r="F31" s="46"/>
-      <c r="G31" s="46"/>
-      <c r="H31" s="46"/>
-      <c r="I31" s="46"/>
-      <c r="J31" s="46"/>
-      <c r="K31" s="46"/>
-      <c r="L31" s="47"/>
+      <c r="C31" s="44"/>
+      <c r="D31" s="44"/>
+      <c r="E31" s="44"/>
+      <c r="F31" s="44"/>
+      <c r="G31" s="44"/>
+      <c r="H31" s="44"/>
+      <c r="I31" s="44"/>
+      <c r="J31" s="44"/>
+      <c r="K31" s="44"/>
+      <c r="L31" s="45"/>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.5">
-      <c r="A32" s="50"/>
-      <c r="B32" s="51"/>
-      <c r="C32" s="51"/>
-      <c r="D32" s="51"/>
-      <c r="E32" s="51"/>
-      <c r="F32" s="51"/>
-      <c r="G32" s="51"/>
-      <c r="H32" s="51"/>
-      <c r="I32" s="51"/>
-      <c r="J32" s="51"/>
-      <c r="K32" s="51"/>
-      <c r="L32" s="52"/>
+      <c r="A32" s="48"/>
+      <c r="B32" s="49"/>
+      <c r="C32" s="49"/>
+      <c r="D32" s="49"/>
+      <c r="E32" s="49"/>
+      <c r="F32" s="49"/>
+      <c r="G32" s="49"/>
+      <c r="H32" s="49"/>
+      <c r="I32" s="49"/>
+      <c r="J32" s="49"/>
+      <c r="K32" s="49"/>
+      <c r="L32" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2005,7 +2089,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr defaultColWidth="20.125" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="14.5" customWidth="1"/>
@@ -2020,17 +2104,17 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="16.149999999999999" thickBot="1" x14ac:dyDescent="0.55000000000000004"/>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.5">
-      <c r="A3" s="57" t="s">
+    <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A3" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="65" t="s">
+      <c r="B3" s="63" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="65" t="s">
+      <c r="C3" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="63" t="s">
+      <c r="D3" s="61" t="s">
         <v>17</v>
       </c>
       <c r="E3" s="9">
@@ -2053,10 +2137,10 @@
       </c>
     </row>
     <row r="4" spans="1:10" ht="31.5" x14ac:dyDescent="0.5">
-      <c r="A4" s="58"/>
-      <c r="B4" s="66"/>
-      <c r="C4" s="66"/>
-      <c r="D4" s="64"/>
+      <c r="A4" s="56"/>
+      <c r="B4" s="64"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="62"/>
       <c r="E4" s="11" t="s">
         <v>18</v>
       </c>
@@ -2077,10 +2161,10 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="58"/>
-      <c r="B5" s="66"/>
-      <c r="C5" s="66"/>
-      <c r="D5" s="64"/>
+      <c r="A5" s="56"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="62"/>
       <c r="E5" s="15" t="s">
         <v>24</v>
       </c>
@@ -2100,36 +2184,52 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A6" s="11"/>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="20" t="s">
+    <row r="6" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="18">
+        <v>4</v>
+      </c>
+      <c r="D6" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="21" t="s">
+      <c r="F6" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="G6" s="21" t="s">
+      <c r="G6" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="H6" s="21" t="s">
+      <c r="H6" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="I6" s="21" t="s">
+      <c r="I6" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J6" s="22" t="s">
+      <c r="J6" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A7" s="11"/>
-      <c r="B7" s="18"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="11" t="s">
+    <row r="7" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="18">
+        <v>4</v>
+      </c>
+      <c r="D7" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F7" s="5" t="s">
@@ -2141,19 +2241,27 @@
       <c r="H7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J7" s="22" t="s">
+      <c r="J7" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A8" s="11"/>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="11" t="s">
+    <row r="8" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="18">
+        <v>4</v>
+      </c>
+      <c r="D8" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F8" s="5" t="s">
@@ -2165,19 +2273,27 @@
       <c r="H8" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J8" s="22" t="s">
+      <c r="J8" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A9" s="11"/>
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="40"/>
-      <c r="E9" s="11" t="s">
+    <row r="9" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="18">
+        <v>4</v>
+      </c>
+      <c r="D9" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E9" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F9" s="5" t="s">
@@ -2189,19 +2305,27 @@
       <c r="H9" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="I9" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J9" s="22" t="s">
+      <c r="J9" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A10" s="11"/>
-      <c r="B10" s="18"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="40"/>
-      <c r="E10" s="11" t="s">
+    <row r="10" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="18">
+        <v>4</v>
+      </c>
+      <c r="D10" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F10" s="5" t="s">
@@ -2213,19 +2337,27 @@
       <c r="H10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="I10" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J10" s="22" t="s">
+      <c r="J10" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A11" s="11"/>
-      <c r="B11" s="18"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="40"/>
-      <c r="E11" s="11" t="s">
+    <row r="11" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="18">
+        <v>4</v>
+      </c>
+      <c r="D11" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F11" s="5" t="s">
@@ -2237,19 +2369,27 @@
       <c r="H11" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J11" s="22" t="s">
+      <c r="J11" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A12" s="11"/>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="11" t="s">
+    <row r="12" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="18">
+        <v>4</v>
+      </c>
+      <c r="D12" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E12" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F12" s="5" t="s">
@@ -2261,19 +2401,27 @@
       <c r="H12" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I12" s="5" t="s">
+      <c r="I12" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J12" s="22" t="s">
+      <c r="J12" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A13" s="11"/>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="40"/>
-      <c r="E13" s="11" t="s">
+    <row r="13" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="18">
+        <v>4</v>
+      </c>
+      <c r="D13" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F13" s="5" t="s">
@@ -2285,19 +2433,27 @@
       <c r="H13" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="I13" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J13" s="22" t="s">
+      <c r="J13" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A14" s="11"/>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="40"/>
-      <c r="E14" s="11" t="s">
+    <row r="14" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="18">
+        <v>4</v>
+      </c>
+      <c r="D14" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E14" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F14" s="5" t="s">
@@ -2309,19 +2465,27 @@
       <c r="H14" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I14" s="5" t="s">
+      <c r="I14" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J14" s="22" t="s">
+      <c r="J14" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A15" s="11"/>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="11" t="s">
+    <row r="15" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="18">
+        <v>4</v>
+      </c>
+      <c r="D15" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E15" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F15" s="5" t="s">
@@ -2333,19 +2497,27 @@
       <c r="H15" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I15" s="5" t="s">
+      <c r="I15" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J15" s="22" t="s">
+      <c r="J15" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A16" s="11"/>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="40"/>
-      <c r="E16" s="11" t="s">
+    <row r="16" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="18">
+        <v>4</v>
+      </c>
+      <c r="D16" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E16" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F16" s="5" t="s">
@@ -2357,19 +2529,27 @@
       <c r="H16" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I16" s="5" t="s">
+      <c r="I16" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J16" s="22" t="s">
+      <c r="J16" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A17" s="11"/>
-      <c r="B17" s="18"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="40"/>
-      <c r="E17" s="11" t="s">
+    <row r="17" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B17" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" s="18">
+        <v>4</v>
+      </c>
+      <c r="D17" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E17" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F17" s="5" t="s">
@@ -2381,19 +2561,27 @@
       <c r="H17" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I17" s="5" t="s">
+      <c r="I17" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J17" s="22" t="s">
+      <c r="J17" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A18" s="11"/>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="40"/>
-      <c r="E18" s="11" t="s">
+    <row r="18" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="18">
+        <v>4</v>
+      </c>
+      <c r="D18" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F18" s="5" t="s">
@@ -2405,19 +2593,27 @@
       <c r="H18" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I18" s="5" t="s">
+      <c r="I18" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J18" s="22" t="s">
+      <c r="J18" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A19" s="11"/>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="40"/>
-      <c r="E19" s="11" t="s">
+    <row r="19" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="18">
+        <v>4</v>
+      </c>
+      <c r="D19" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E19" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F19" s="5" t="s">
@@ -2429,19 +2625,27 @@
       <c r="H19" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I19" s="5" t="s">
+      <c r="I19" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J19" s="22" t="s">
+      <c r="J19" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A20" s="11"/>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="40"/>
-      <c r="E20" s="11" t="s">
+    <row r="20" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A20" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="18">
+        <v>4</v>
+      </c>
+      <c r="D20" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E20" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F20" s="5" t="s">
@@ -2453,19 +2657,27 @@
       <c r="H20" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I20" s="5" t="s">
+      <c r="I20" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J20" s="22" t="s">
+      <c r="J20" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A21" s="11"/>
-      <c r="B21" s="18"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="40"/>
-      <c r="E21" s="11" t="s">
+    <row r="21" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A21" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="18">
+        <v>4</v>
+      </c>
+      <c r="D21" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E21" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F21" s="5" t="s">
@@ -2477,19 +2689,27 @@
       <c r="H21" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I21" s="5" t="s">
+      <c r="I21" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J21" s="22" t="s">
+      <c r="J21" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A22" s="11"/>
-      <c r="B22" s="18"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="40"/>
-      <c r="E22" s="11" t="s">
+    <row r="22" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A22" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" s="18">
+        <v>4</v>
+      </c>
+      <c r="D22" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E22" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F22" s="5" t="s">
@@ -2501,19 +2721,27 @@
       <c r="H22" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I22" s="5" t="s">
+      <c r="I22" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J22" s="22" t="s">
+      <c r="J22" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A23" s="11"/>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="40"/>
-      <c r="E23" s="11" t="s">
+    <row r="23" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A23" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="18">
+        <v>4</v>
+      </c>
+      <c r="D23" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E23" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F23" s="5" t="s">
@@ -2525,19 +2753,27 @@
       <c r="H23" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I23" s="5" t="s">
+      <c r="I23" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J23" s="22" t="s">
+      <c r="J23" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A24" s="11"/>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="40"/>
-      <c r="E24" s="11" t="s">
+    <row r="24" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A24" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B24" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C24" s="18">
+        <v>4</v>
+      </c>
+      <c r="D24" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E24" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F24" s="5" t="s">
@@ -2549,19 +2785,27 @@
       <c r="H24" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I24" s="5" t="s">
+      <c r="I24" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J24" s="22" t="s">
+      <c r="J24" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A25" s="11"/>
-      <c r="B25" s="18"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="40"/>
-      <c r="E25" s="11" t="s">
+    <row r="25" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A25" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" s="18">
+        <v>4</v>
+      </c>
+      <c r="D25" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E25" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F25" s="5" t="s">
@@ -2573,19 +2817,27 @@
       <c r="H25" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I25" s="5" t="s">
+      <c r="I25" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J25" s="22" t="s">
+      <c r="J25" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A26" s="11"/>
-      <c r="B26" s="18"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="40"/>
-      <c r="E26" s="11" t="s">
+    <row r="26" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A26" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="C26" s="18">
+        <v>4</v>
+      </c>
+      <c r="D26" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E26" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F26" s="5" t="s">
@@ -2597,19 +2849,27 @@
       <c r="H26" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I26" s="5" t="s">
+      <c r="I26" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J26" s="22" t="s">
+      <c r="J26" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A27" s="11"/>
-      <c r="B27" s="18"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="40"/>
-      <c r="E27" s="11" t="s">
+    <row r="27" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A27" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" s="18">
+        <v>4</v>
+      </c>
+      <c r="D27" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E27" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F27" s="5" t="s">
@@ -2621,19 +2881,27 @@
       <c r="H27" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I27" s="5" t="s">
+      <c r="I27" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J27" s="22" t="s">
+      <c r="J27" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A28" s="11"/>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="40"/>
-      <c r="E28" s="11" t="s">
+    <row r="28" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A28" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C28" s="18">
+        <v>4</v>
+      </c>
+      <c r="D28" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E28" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F28" s="5" t="s">
@@ -2645,19 +2913,27 @@
       <c r="H28" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I28" s="5" t="s">
+      <c r="I28" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J28" s="22" t="s">
+      <c r="J28" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A29" s="11"/>
-      <c r="B29" s="18"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="40"/>
-      <c r="E29" s="11" t="s">
+    <row r="29" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A29" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B29" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" s="18">
+        <v>4</v>
+      </c>
+      <c r="D29" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E29" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F29" s="5" t="s">
@@ -2669,21 +2945,27 @@
       <c r="H29" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I29" s="5" t="s">
+      <c r="I29" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J29" s="22" t="s">
+      <c r="J29" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B30" s="18"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="40"/>
-      <c r="E30" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="C30" s="18">
+        <v>4</v>
+      </c>
+      <c r="D30" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E30" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F30" s="5" t="s">
@@ -2695,19 +2977,27 @@
       <c r="H30" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I30" s="5" t="s">
+      <c r="I30" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J30" s="22" t="s">
+      <c r="J30" s="21" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="47.25" x14ac:dyDescent="0.5">
-      <c r="A31" s="11"/>
-      <c r="B31" s="18"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="40"/>
-      <c r="E31" s="11" t="s">
+    <row r="31" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A31" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="C31" s="18">
+        <v>4</v>
+      </c>
+      <c r="D31" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E31" s="15" t="s">
         <v>24</v>
       </c>
       <c r="F31" s="5" t="s">
@@ -2719,34 +3009,74 @@
       <c r="H31" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I31" s="5" t="s">
+      <c r="I31" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J31" s="22" t="s">
+      <c r="J31" s="21" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="15"/>
-      <c r="B32" s="39"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="41"/>
+      <c r="A32" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="B32" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="C32" s="18">
+        <v>4</v>
+      </c>
+      <c r="D32" s="39" t="s">
+        <v>47</v>
+      </c>
       <c r="E32" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="F32" s="16" t="s">
+      <c r="F32" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="G32" s="16" t="s">
+      <c r="G32" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="H32" s="16" t="s">
+      <c r="H32" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I32" s="16" t="s">
+      <c r="I32" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="J32" s="22" t="s">
+      <c r="J32" s="21" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="47.65" thickBot="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A33" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="B33" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="C33" s="18">
+        <v>4</v>
+      </c>
+      <c r="D33" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="F33" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="G33" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="H33" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="I33" s="65" t="s">
+        <v>28</v>
+      </c>
+      <c r="J33" s="21" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2757,33 +3087,27 @@
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="A3:A5"/>
   </mergeCells>
-  <conditionalFormatting sqref="E6:J32">
+  <conditionalFormatting sqref="F6:J33">
     <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
-      <formula>$C6=E$3</formula>
+      <formula>$C6=F$3</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C6:C32" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C6:C33" xr:uid="{26B80383-77F6-4F19-9480-F27CEB49F33A}">
       <formula1>$E$3:$J$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000002000000}">
-          <x14:formula1>
-            <xm:f>'Team and Self Assessment'!$C$10:$C$17</xm:f>
-          </x14:formula1>
-          <xm:sqref>B6:B32</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005836243B3C47804EAF5FFDD9F066FCC7" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9d21ddf3f0b128e39c9d770c8c903166">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b0326308c339679ad994635f2c691325" ns2:_="">
     <xsd:import namespace="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
@@ -2967,12 +3291,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2983,6 +3301,22 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23B77F7C-EE47-4FBD-B078-6536C1487A1E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3000,22 +3334,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D8D82CB-2E6F-4A14-B6B4-DFDD1BBD70FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="a1e3ca88-8ae5-4fd0-ba37-40ce669fcbb0"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F61419B8-A98A-41CD-95EE-48A4F975B8D1}">
   <ds:schemaRefs>

</xml_diff>